<commit_message>
[WIP] int? 타입 다 List<int> 로 변환중
</commit_message>
<xml_diff>
--- a/Assets/Data/Source/Excel/2026_StellarFoodship_DataTable.xlsx
+++ b/Assets/Data/Source/Excel/2026_StellarFoodship_DataTable.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="148">
   <si>
     <t>id</t>
   </si>
@@ -121,19 +121,22 @@
     <t>cookwareTypeString</t>
   </si>
   <si>
+    <t>cookTypeIconPath</t>
+  </si>
+  <si>
     <t>탄 조리품</t>
   </si>
   <si>
     <t>burntProcessed</t>
   </si>
   <si>
+    <t>Pan</t>
+  </si>
+  <si>
     <t>외계 살사</t>
   </si>
   <si>
     <t>alienSalsa</t>
-  </si>
-  <si>
-    <t>Pan</t>
   </si>
   <si>
     <t>우주 필레</t>
@@ -1145,8 +1148,9 @@
     <col customWidth="1" min="2" max="2" width="19.63"/>
     <col customWidth="1" min="3" max="3" width="16.63"/>
     <col customWidth="1" min="8" max="8" width="16.25"/>
-    <col customWidth="1" min="9" max="9" width="34.75"/>
-    <col customWidth="1" min="10" max="10" width="35.75"/>
+    <col customWidth="1" min="9" max="9" width="36.13"/>
+    <col customWidth="1" min="10" max="10" width="34.75"/>
+    <col customWidth="1" min="11" max="11" width="35.75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1175,9 +1179,12 @@
         <v>34</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1186,22 +1193,36 @@
         <v>100.0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="3"/>
+        <v>37</v>
+      </c>
+      <c r="D2" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="E2" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="F2" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="G2" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>38</v>
+      </c>
       <c r="I2" s="4" t="str">
-        <f t="shared" ref="I2:I11" si="1">"Icons/CookedIngredient/" &amp; C2</f>
+        <f t="shared" ref="I2:I11" si="1">"Icons/CookType/" &amp; H2</f>
+        <v>Icons/CookType/Pan</v>
+      </c>
+      <c r="J2" s="4" t="str">
+        <f t="shared" ref="J2:J11" si="2">"Icons/CookedIngredient/" &amp; C2</f>
         <v>Icons/CookedIngredient/burntProcessed</v>
       </c>
-      <c r="J2" s="6" t="str">
-        <f t="shared" ref="J2:J11" si="2">"Model/CookedIngredient/" &amp; C2</f>
+      <c r="K2" s="6" t="str">
+        <f t="shared" ref="K2:K11" si="3">"Model/CookedIngredient/" &amp; C2</f>
         <v>Model/CookedIngredient/burntProcessed</v>
       </c>
     </row>
@@ -1210,13 +1231,17 @@
         <v>101.0</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
+        <v>40</v>
+      </c>
+      <c r="D3" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="F3" s="5">
         <v>0.0</v>
       </c>
@@ -1224,14 +1249,18 @@
         <v>1.0</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I3" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/Pan</v>
+      </c>
+      <c r="J3" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/alienSalsa</v>
       </c>
-      <c r="J3" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K3" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/alienSalsa</v>
       </c>
     </row>
@@ -1240,26 +1269,36 @@
         <v>102.0</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+        <v>42</v>
+      </c>
+      <c r="D4" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="F4" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="G4" s="5">
         <v>2.0</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I4" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/Steamer</v>
+      </c>
+      <c r="J4" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/plasmaFillet</v>
       </c>
-      <c r="J4" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K4" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/plasmaFillet</v>
       </c>
     </row>
@@ -1268,12 +1307,14 @@
         <v>103.0</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="5"/>
+        <v>45</v>
+      </c>
+      <c r="D5" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="E5" s="5">
         <v>0.0</v>
       </c>
@@ -1284,14 +1325,18 @@
         <v>3.0</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I5" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/Pot</v>
+      </c>
+      <c r="J5" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/plasmaNeonStew</v>
       </c>
-      <c r="J5" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K5" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/plasmaNeonStew</v>
       </c>
     </row>
@@ -1300,12 +1345,14 @@
         <v>104.0</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="D6" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="E6" s="5">
         <v>0.0</v>
       </c>
@@ -1316,14 +1363,18 @@
         <v>3.0</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I6" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/MixerCup</v>
+      </c>
+      <c r="J6" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/neonSalad</v>
       </c>
-      <c r="J6" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K6" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/neonSalad</v>
       </c>
     </row>
@@ -1332,13 +1383,17 @@
         <v>105.0</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+        <v>51</v>
+      </c>
+      <c r="D7" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E7" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="F7" s="5">
         <v>7.0</v>
       </c>
@@ -1346,14 +1401,18 @@
         <v>8.0</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I7" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/Pan</v>
+      </c>
+      <c r="J7" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/Blackholeomelet</v>
       </c>
-      <c r="J7" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K7" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/Blackholeomelet</v>
       </c>
     </row>
@@ -1362,13 +1421,17 @@
         <v>106.0</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+        <v>53</v>
+      </c>
+      <c r="D8" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E8" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="F8" s="5">
         <v>6.0</v>
       </c>
@@ -1376,14 +1439,18 @@
         <v>9.0</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I8" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/Steamer</v>
+      </c>
+      <c r="J8" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/starCreamRisotto</v>
       </c>
-      <c r="J8" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K8" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/starCreamRisotto</v>
       </c>
     </row>
@@ -1392,13 +1459,17 @@
         <v>107.0</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="D9" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E9" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="F9" s="5">
         <v>5.0</v>
       </c>
@@ -1406,14 +1477,18 @@
         <v>8.0</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I9" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/Steamer</v>
+      </c>
+      <c r="J9" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/lavaBlackholeSteam</v>
       </c>
-      <c r="J9" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K9" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/lavaBlackholeSteam</v>
       </c>
     </row>
@@ -1422,26 +1497,36 @@
         <v>108.0</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
+        <v>57</v>
+      </c>
+      <c r="D10" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E10" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="F10" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="G10" s="5">
         <v>4.0</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I10" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/Pan</v>
+      </c>
+      <c r="J10" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/cosmicRiceBowl</v>
       </c>
-      <c r="J10" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K10" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/cosmicRiceBowl</v>
       </c>
     </row>
@@ -1450,13 +1535,17 @@
         <v>109.0</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
+        <v>59</v>
+      </c>
+      <c r="D11" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="E11" s="8">
+        <v>-1.0</v>
+      </c>
       <c r="F11" s="8">
         <v>3.0</v>
       </c>
@@ -1464,14 +1553,18 @@
         <v>9.0</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I11" s="4" t="str">
         <f t="shared" si="1"/>
+        <v>Icons/CookType/Pan</v>
+      </c>
+      <c r="J11" s="4" t="str">
+        <f t="shared" si="2"/>
         <v>Icons/CookedIngredient/friedNeonJelly</v>
       </c>
-      <c r="J11" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="K11" s="6" t="str">
+        <f t="shared" si="3"/>
         <v>Model/CookedIngredient/friedNeonJelly</v>
       </c>
     </row>
@@ -7438,7 +7531,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -7456,7 +7549,7 @@
         <v>33</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>34</v>
@@ -7473,20 +7566,28 @@
         <v>200.0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
+        <v>63</v>
+      </c>
+      <c r="D2" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="E2" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="F2" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="G2" s="8">
+        <v>-1.0</v>
+      </c>
       <c r="H2" s="3">
         <v>-50.0</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J2" s="4" t="str">
         <f t="shared" ref="J2:J11" si="1">"Icons/Dish/" &amp; C2</f>
@@ -7502,14 +7603,20 @@
         <v>201.0</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
+        <v>40</v>
+      </c>
+      <c r="D3" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="F3" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="G3" s="5">
         <v>101.0</v>
       </c>
@@ -7517,7 +7624,7 @@
         <v>30.0</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J3" s="4" t="str">
         <f t="shared" si="1"/>
@@ -7533,14 +7640,20 @@
         <v>202.0</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+        <v>42</v>
+      </c>
+      <c r="D4" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="F4" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="G4" s="5">
         <v>102.0</v>
       </c>
@@ -7548,7 +7661,7 @@
         <v>20.0</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J4" s="3" t="str">
         <f t="shared" si="1"/>
@@ -7564,14 +7677,20 @@
         <v>203.0</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
+        <v>45</v>
+      </c>
+      <c r="D5" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E5" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="F5" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="G5" s="5">
         <v>103.0</v>
       </c>
@@ -7579,7 +7698,7 @@
         <v>80.0</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J5" s="4" t="str">
         <f t="shared" si="1"/>
@@ -7595,14 +7714,20 @@
         <v>204.0</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="D6" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E6" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="F6" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="G6" s="5">
         <v>104.0</v>
       </c>
@@ -7610,7 +7735,7 @@
         <v>80.0</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J6" s="3" t="str">
         <f t="shared" si="1"/>
@@ -7626,13 +7751,17 @@
         <v>205.0</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+        <v>51</v>
+      </c>
+      <c r="D7" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E7" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="F7" s="5">
         <v>105.0</v>
       </c>
@@ -7643,7 +7772,7 @@
         <v>80.0</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J7" s="4" t="str">
         <f t="shared" si="1"/>
@@ -7659,13 +7788,17 @@
         <v>206.0</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+        <v>53</v>
+      </c>
+      <c r="D8" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E8" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="F8" s="5">
         <v>106.0</v>
       </c>
@@ -7676,7 +7809,7 @@
         <v>80.0</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J8" s="3" t="str">
         <f t="shared" si="1"/>
@@ -7692,14 +7825,20 @@
         <v>207.0</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="D9" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="E9" s="5">
+        <v>-1.0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="G9" s="5">
         <v>107.0</v>
       </c>
@@ -7707,7 +7846,7 @@
         <v>30.0</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J9" s="4" t="str">
         <f t="shared" si="1"/>
@@ -7723,12 +7862,14 @@
         <v>208.0</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" s="5"/>
+        <v>57</v>
+      </c>
+      <c r="D10" s="5">
+        <v>-1.0</v>
+      </c>
       <c r="E10" s="5">
         <v>101.0</v>
       </c>
@@ -7742,7 +7883,7 @@
         <v>100.0</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J10" s="3" t="str">
         <f t="shared" si="1"/>
@@ -7758,14 +7899,20 @@
         <v>209.0</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
+        <v>59</v>
+      </c>
+      <c r="D11" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="E11" s="8">
+        <v>-1.0</v>
+      </c>
+      <c r="F11" s="8">
+        <v>-1.0</v>
+      </c>
       <c r="G11" s="8">
         <v>109.0</v>
       </c>
@@ -7773,7 +7920,7 @@
         <v>30.0</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J11" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13742,19 +13889,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>5</v>
@@ -13765,19 +13912,19 @@
         <v>0.0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E2" s="3">
         <v>1.0</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G2" s="4" t="str">
         <f t="shared" ref="G2:G27" si="1">"Icons/Achievement/" &amp; C2</f>
@@ -13789,10 +13936,10 @@
         <v>1.0</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D3" s="4" t="str">
         <f t="shared" ref="D3:D11" si="2">B3 &amp; "를 완성하세요."</f>
@@ -13802,7 +13949,7 @@
         <v>1.0</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G3" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13814,10 +13961,10 @@
         <v>2.0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D4" s="4" t="str">
         <f t="shared" si="2"/>
@@ -13827,7 +13974,7 @@
         <v>1.0</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G4" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13839,10 +13986,10 @@
         <v>3.0</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D5" s="4" t="str">
         <f t="shared" si="2"/>
@@ -13852,7 +13999,7 @@
         <v>1.0</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G5" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13864,10 +14011,10 @@
         <v>4.0</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D6" s="4" t="str">
         <f t="shared" si="2"/>
@@ -13877,7 +14024,7 @@
         <v>1.0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G6" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13889,10 +14036,10 @@
         <v>5.0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D7" s="4" t="str">
         <f t="shared" si="2"/>
@@ -13902,7 +14049,7 @@
         <v>1.0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G7" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13914,10 +14061,10 @@
         <v>6.0</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D8" s="4" t="str">
         <f t="shared" si="2"/>
@@ -13927,7 +14074,7 @@
         <v>1.0</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G8" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13939,10 +14086,10 @@
         <v>7.0</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D9" s="4" t="str">
         <f t="shared" si="2"/>
@@ -13952,7 +14099,7 @@
         <v>1.0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G9" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13964,10 +14111,10 @@
         <v>8.0</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D10" s="4" t="str">
         <f t="shared" si="2"/>
@@ -13977,7 +14124,7 @@
         <v>1.0</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G10" s="4" t="str">
         <f t="shared" si="1"/>
@@ -13989,10 +14136,10 @@
         <v>9.0</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D11" s="4" t="str">
         <f t="shared" si="2"/>
@@ -14002,7 +14149,7 @@
         <v>1.0</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G11" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14014,19 +14161,19 @@
         <v>10.0</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E12" s="3">
         <v>1.0</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G12" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14038,19 +14185,19 @@
         <v>11.0</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E13" s="3">
         <v>1.0</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G13" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14062,19 +14209,19 @@
         <v>12.0</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E14" s="3">
         <v>1.0</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G14" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14086,19 +14233,19 @@
         <v>13.0</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E15" s="3">
         <v>1.0</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G15" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14110,19 +14257,19 @@
         <v>14.0</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E16" s="3">
         <v>1.0</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G16" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14134,19 +14281,19 @@
         <v>15.0</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E17" s="3">
         <v>1.0</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G17" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14158,19 +14305,19 @@
         <v>16.0</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E18" s="3">
         <v>1.0</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G18" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14182,19 +14329,19 @@
         <v>17.0</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E19" s="3">
         <v>1.0</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G19" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14206,19 +14353,19 @@
         <v>18.0</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E20" s="3">
         <v>1.0</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G20" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14230,19 +14377,19 @@
         <v>19.0</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E21" s="3">
         <v>100.0</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G21" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14254,19 +14401,19 @@
         <v>20.0</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E22" s="3">
         <v>500.0</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G22" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14278,19 +14425,19 @@
         <v>21.0</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E23" s="3">
         <v>1000.0</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G23" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14302,19 +14449,19 @@
         <v>22.0</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E24" s="3">
         <v>1.0</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G24" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14326,19 +14473,19 @@
         <v>23.0</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E25" s="3">
         <v>1.0</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G25" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14350,19 +14497,19 @@
         <v>24.0</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E26" s="3">
         <v>1.0</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G26" s="4" t="str">
         <f t="shared" si="1"/>
@@ -14374,19 +14521,19 @@
         <v>25.0</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E27" s="3">
         <v>1.0</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G27" s="4" t="str">
         <f t="shared" si="1"/>

</xml_diff>